<commit_message>
Generar presupuesto P-2026-0050 nave industrial Alaior (estructura, paneles y carpinteria exterior)
</commit_message>
<xml_diff>
--- a/presupuestos/Presupuesto_Alaior_Estructura_Paneles_Carpinterias.xlsx
+++ b/presupuestos/Presupuesto_Alaior_Estructura_Paneles_Carpinterias.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen General" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1.3 Estructura Metálica" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1.8 Conteo Carpinterías" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2.0 Paneles y Cubierta" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Resumen General" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="1.3 Estructura Metálica" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="1.8 Conteo Carpinterías" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="2.0 Paneles y Cubierta" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="B2:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -568,7 +568,6 @@
     <col width="15" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -583,7 +582,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -751,17 +749,20 @@
         </is>
       </c>
       <c r="E10" s="11" t="n">
-        <v>938</v>
+        <v>25</v>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
           <t>Rigidizadores y arriostramientos de nave</t>
         </is>
       </c>
-      <c r="G10" s="12" t="n"/>
-      <c r="H10" s="12" t="n"/>
-    </row>
-    <row r="11"/>
+      <c r="G10" s="12" t="n">
+        <v>19650</v>
+      </c>
+      <c r="H10" s="12" t="n">
+        <v>19650</v>
+      </c>
+    </row>
     <row r="12">
       <c r="B12" s="5" t="inlineStr">
         <is>
@@ -850,7 +851,6 @@
         <v>6750</v>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="B16" s="5" t="inlineStr">
         <is>
@@ -906,7 +906,7 @@
         </is>
       </c>
       <c r="G17" s="14" t="n">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="H17" s="14">
         <f>E17*G17</f>
@@ -938,7 +938,7 @@
         </is>
       </c>
       <c r="G18" s="14" t="n">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="H18" s="14">
         <f>E18*G18</f>
@@ -970,14 +970,13 @@
         </is>
       </c>
       <c r="G19" s="14" t="n">
-        <v>176</v>
+        <v>165</v>
       </c>
       <c r="H19" s="14">
         <f>E19*G19</f>
         <v/>
       </c>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="F21" s="15" t="inlineStr">
         <is>
@@ -1000,7 +999,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="B2:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1014,7 +1013,6 @@
     <col width="20" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -1029,7 +1027,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="B5" s="4" t="inlineStr">
         <is>
@@ -1241,7 +1238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="B2:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1258,7 +1255,6 @@
     <col width="28" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -1273,7 +1269,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="B5" s="4" t="inlineStr">
         <is>
@@ -1711,7 +1706,7 @@
       </c>
       <c r="I14" s="9" t="inlineStr">
         <is>
-          <t>Marco aluminio anodizado + policarbonato termoformado + babeta</t>
+          <t>Marco aluminio anodizado + policarbonato (Presupuestado en cap. 2.3 Lucernarios)</t>
         </is>
       </c>
       <c r="J14" s="9" t="inlineStr">
@@ -1720,11 +1715,10 @@
         </is>
       </c>
       <c r="K14" s="14" t="n">
-        <v>250</v>
-      </c>
-      <c r="L14" s="14">
-        <f>D14*K14</f>
-        <v/>
+        <v>0</v>
+      </c>
+      <c r="L14" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -1876,7 +1870,6 @@
         <v/>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="C20" s="17" t="inlineStr">
         <is>
@@ -1907,7 +1900,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="B2:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1922,7 +1915,6 @@
     <col width="58" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -1937,7 +1929,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="B5" s="4" t="inlineStr">
         <is>
@@ -2002,7 +1993,7 @@
         </is>
       </c>
       <c r="E6" s="11" t="n">
-        <v>346.87</v>
+        <v>120</v>
       </c>
       <c r="F6" s="14" t="n">
         <v>110</v>
@@ -2044,7 +2035,7 @@
         </is>
       </c>
       <c r="E7" s="11" t="n">
-        <v>711.75</v>
+        <v>165</v>
       </c>
       <c r="F7" s="14" t="n">
         <v>175</v>
@@ -2086,7 +2077,7 @@
         </is>
       </c>
       <c r="E8" s="11" t="n">
-        <v>15</v>
+        <v>165</v>
       </c>
       <c r="F8" s="14" t="n">
         <v>176</v>

</xml_diff>